<commit_message>
update offline prompt and CLI
</commit_message>
<xml_diff>
--- a/artifacts/output/test1_output.xlsx
+++ b/artifacts/output/test1_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Output" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,12 +28,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF0000"/>
+        <bgColor rgb="00FF0000"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -48,9 +54,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -416,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D276"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,6 +461,9 @@
       <c r="C2" t="n">
         <v>106.11</v>
       </c>
+      <c r="D2" t="n">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -466,6 +477,9 @@
       <c r="C3" t="n">
         <v>43.62</v>
       </c>
+      <c r="D3" t="n">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -495,7 +509,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -569,6 +583,9 @@
       <c r="C9" t="n">
         <v>116.58</v>
       </c>
+      <c r="D9" t="n">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -762,6 +779,9 @@
       <c r="C20" t="n">
         <v>107.96</v>
       </c>
+      <c r="D20" t="n">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -791,7 +811,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v/>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -829,6 +849,9 @@
       <c r="C24" t="n">
         <v>115.04</v>
       </c>
+      <c r="D24" t="n">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -878,6 +901,9 @@
       <c r="C27" t="n">
         <v>102.98</v>
       </c>
+      <c r="D27" t="n">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -954,34 +980,28 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+          <t>Total Spending (£)</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>2023.75</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Total Spending (£)</t>
+          <t>Average Daily Spending (£)</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2023.75</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Average Daily Spending (£)</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>67.45833333333333</v>
-      </c>
+        <v>72.27678571428571</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="n"/>
+      <c r="B276" s="3" t="n"/>
+      <c r="C276" s="3" t="n"/>
+      <c r="D276" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fixed validation result parsing bug
</commit_message>
<xml_diff>
--- a/artifacts/output/test1_output.xlsx
+++ b/artifacts/output/test1_output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Output" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Output" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D276"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,9 +461,6 @@
       <c r="C2" t="n">
         <v>106.11</v>
       </c>
-      <c r="D2" t="n">
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -477,9 +474,6 @@
       <c r="C3" t="n">
         <v>43.62</v>
       </c>
-      <c r="D3" t="n">
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -509,7 +503,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -572,20 +566,18 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>45969</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="3" t="n">
         <v>116.58</v>
       </c>
-      <c r="D9" t="n">
-        <v/>
-      </c>
+      <c r="D9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -779,9 +771,6 @@
       <c r="C20" t="n">
         <v>107.96</v>
       </c>
-      <c r="D20" t="n">
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -849,9 +838,6 @@
       <c r="C24" t="n">
         <v>115.04</v>
       </c>
-      <c r="D24" t="n">
-        <v/>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -901,9 +887,6 @@
       <c r="C27" t="n">
         <v>102.98</v>
       </c>
-      <c r="D27" t="n">
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -980,28 +963,34 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Total Spending (£)</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>2023.75</v>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Total Spending (£)</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2023.75</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Average Daily Spending (£)</t>
         </is>
       </c>
-      <c r="B34" t="n">
-        <v>72.27678571428571</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" s="3" t="n"/>
-      <c r="B276" s="3" t="n"/>
-      <c r="C276" s="3" t="n"/>
-      <c r="D276" s="3" t="n"/>
+      <c r="B35" t="n">
+        <v>69.78448275862068</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
improve QA diagnose alignment and clarify execution context handling
</commit_message>
<xml_diff>
--- a/artifacts/output/test1_output.xlsx
+++ b/artifacts/output/test1_output.xlsx
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -811,7 +811,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v/>
+        <v>0</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -992,7 +992,7 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>72.28</v>
+        <v>67.45999999999999</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
refactor(backend): unify LLM retry, remove legacy execution path, enforce Stage inheritance
</commit_message>
<xml_diff>
--- a/artifacts/output/test1_output.xlsx
+++ b/artifacts/output/test1_output.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,9 +461,7 @@
       <c r="C2" t="n">
         <v>106.11</v>
       </c>
-      <c r="D2" t="n">
-        <v/>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -477,9 +475,7 @@
       <c r="C3" t="n">
         <v>43.62</v>
       </c>
-      <c r="D3" t="n">
-        <v/>
-      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
@@ -583,9 +579,7 @@
       <c r="C9" s="3" t="n">
         <v>116.58</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v/>
-      </c>
+      <c r="D9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
@@ -779,9 +773,7 @@
       <c r="C20" t="n">
         <v>107.96</v>
       </c>
-      <c r="D20" t="n">
-        <v/>
-      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
@@ -849,9 +841,7 @@
       <c r="C24" t="n">
         <v>115.04</v>
       </c>
-      <c r="D24" t="n">
-        <v/>
-      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
@@ -901,9 +891,7 @@
       <c r="C27" t="n">
         <v>102.98</v>
       </c>
-      <c r="D27" t="n">
-        <v/>
-      </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
@@ -977,29 +965,29 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>Total Daily Spending (£)</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B33" t="n">
         <v>2023.75</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Average Daily Spending (£)</t>
         </is>
       </c>
-      <c r="E32" t="n">
+      <c r="E33" t="n">
         <v>67.45999999999999</v>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>Max Daily Spending (£)</t>
         </is>
       </c>
-      <c r="H32" t="n">
+      <c r="H33" t="n">
         <v>116.58</v>
       </c>
     </row>

</xml_diff>